<commit_message>
Add invoice and packing-list numbers to HS summary sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MbbRpLM3rWRDviiDxBw8zw
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Hitachi_Energy_CZ26801003.xlsx
+++ b/output/HS_Code_Summary_Hitachi_Energy_CZ26801003.xlsx
@@ -523,22 +523,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1" ht="42" customHeight="1">
+    <row r="1" ht="48" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>HS kód</t>
@@ -556,35 +558,45 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Faktura č.</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Packing list / dodací list č.</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Celkové množství (ks)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Čistá hmotnost (kg)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Hrubá hmotnost (kg)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Hodnota CHF</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Hodnota CZK</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Příznak</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Poznámka / CBAM / Antidumping / Preferenční původ</t>
         </is>
@@ -606,23 +618,33 @@
           <t>CZ</t>
         </is>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>810678840 + 810678891</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>0923634579 + 0923705937</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="n">
         <v>290</v>
       </c>
-      <c r="E2" s="5" t="n">
+      <c r="G2" s="5" t="n">
         <v>498</v>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="H2" s="5" t="n">
         <v>524</v>
       </c>
-      <c r="G2" s="6" t="n">
+      <c r="I2" s="6" t="n">
         <v>154600</v>
       </c>
-      <c r="H2" s="6" t="n">
+      <c r="J2" s="6" t="n">
         <v>4061187.4</v>
       </c>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>Sloučeny 2 položky faktur (810678840 + 810678891) pod stejný HS 85413000. CBAM: NEPODLÉHÁ (polovodiče nejsou zboží CBAM). Antidumping: neuplatňuje se (původ CZ/EU).</t>
         </is>
@@ -644,27 +666,37 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D3" s="9" t="n">
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>810678841</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>0923634952</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="E3" s="10" t="n">
+      <c r="G3" s="10" t="n">
         <v>11.2</v>
       </c>
-      <c r="F3" s="10" t="n">
+      <c r="H3" s="10" t="n">
         <v>11.2</v>
       </c>
-      <c r="G3" s="11" t="n">
+      <c r="I3" s="11" t="n">
         <v>4172</v>
       </c>
-      <c r="H3" s="11" t="n">
+      <c r="J3" s="11" t="n">
         <v>109594.27</v>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="K3" s="7" t="inlineStr">
         <is>
           <t>POZOR</t>
         </is>
       </c>
-      <c r="J3" s="8" t="inlineStr">
+      <c r="L3" s="8" t="inlineStr">
         <is>
           <t>HS kód i země původu CHYBÍ na faktuře 810678841 i dodacím listu 923634952. HS 85411000 převzat z e-mailu M. Bardy. Původ nutno doplnit/ověřit (pravděpodobně CZ). CBAM: NEPODLÉHÁ. Antidumping: neuplatňuje se.</t>
         </is>
@@ -678,23 +710,25 @@
       </c>
       <c r="B4" s="13" t="inlineStr"/>
       <c r="C4" s="12" t="inlineStr"/>
-      <c r="D4" s="14" t="n">
+      <c r="D4" s="13" t="inlineStr"/>
+      <c r="E4" s="13" t="inlineStr"/>
+      <c r="F4" s="14" t="n">
         <v>297</v>
       </c>
-      <c r="E4" s="15" t="n">
+      <c r="G4" s="15" t="n">
         <v>509.2</v>
       </c>
-      <c r="F4" s="15" t="n">
+      <c r="H4" s="15" t="n">
         <v>535.2</v>
       </c>
-      <c r="G4" s="16" t="n">
+      <c r="I4" s="16" t="n">
         <v>158772</v>
       </c>
-      <c r="H4" s="16" t="n">
+      <c r="J4" s="16" t="n">
         <v>4170781.67</v>
       </c>
-      <c r="I4" s="12" t="inlineStr"/>
-      <c r="J4" s="13" t="inlineStr"/>
+      <c r="K4" s="12" t="inlineStr"/>
+      <c r="L4" s="13" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="17" t="inlineStr">

</xml_diff>